<commit_message>
Add `user7` to IC reference file land details query
</commit_message>
<xml_diff>
--- a/dbt/export/templates/qc.vw_ic_reference_all_non_res_land_details.xlsx
+++ b/dbt/export/templates/qc.vw_ic_reference_all_non_res_land_details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jecochr\Downloads\ic_reference_templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jecochr\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8486AD18-01AC-4EBC-A245-C5EE5F785EF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{490405C4-8E17-4245-ACFE-5C30671C954F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43605" yWindow="3615" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Query Results" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="31">
   <si>
     <t>PARDAT</t>
   </si>
@@ -110,6 +110,9 @@
   </si>
   <si>
     <t>OSIZE</t>
+  </si>
+  <si>
+    <t>Incentive Control Number</t>
   </si>
 </sst>
 </file>
@@ -476,10 +479,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AC2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -564,8 +567,11 @@
       <c r="AB1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="AC1" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -649,6 +655,9 @@
       </c>
       <c r="AB2" s="1" t="s">
         <v>29</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add `land.user7` to IC reference query and fix unexpected formula bug (#1084)
* Add `user7` to IC reference file land details query

* Cast values that start with "=" to string to prevent unexpected formulae in `export_models`
</commit_message>
<xml_diff>
--- a/dbt/export/templates/qc.vw_ic_reference_all_non_res_land_details.xlsx
+++ b/dbt/export/templates/qc.vw_ic_reference_all_non_res_land_details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jecochr\Downloads\ic_reference_templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jecochr\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8486AD18-01AC-4EBC-A245-C5EE5F785EF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{490405C4-8E17-4245-ACFE-5C30671C954F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43605" yWindow="3615" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Query Results" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="31">
   <si>
     <t>PARDAT</t>
   </si>
@@ -110,6 +110,9 @@
   </si>
   <si>
     <t>OSIZE</t>
+  </si>
+  <si>
+    <t>Incentive Control Number</t>
   </si>
 </sst>
 </file>
@@ -476,10 +479,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AC2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -564,8 +567,11 @@
       <c r="AB1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="AC1" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -649,6 +655,9 @@
       </c>
       <c r="AB2" s="1" t="s">
         <v>29</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>